<commit_message>
Practicando Excel y haciendo evidencia de liz
</commit_message>
<xml_diff>
--- a/chamba/Excel_Practice/121 - Converting data.xlsx
+++ b/chamba/Excel_Practice/121 - Converting data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alex_\Em1Repo\chamba\Excel_Practice\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F202F25F-AF5E-494E-A1B3-0EFDF4E990B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F33E329-E807-4735-8A6F-B02FCE358F68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{EC2FC403-3BD3-48C3-93CE-3A4A505B5772}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{EC2FC403-3BD3-48C3-93CE-3A4A505B5772}"/>
   </bookViews>
   <sheets>
     <sheet name="Supplier Invoice Statement" sheetId="2" r:id="rId1"/>
@@ -7647,7 +7647,7 @@
       </c>
       <c r="B2" s="15">
         <f ca="1">TODAY()</f>
-        <v>46301</v>
+        <v>46303</v>
       </c>
       <c r="D2"/>
       <c r="E2"/>
@@ -7914,15 +7914,15 @@
       </c>
       <c r="Q8" s="15">
         <f ca="1">TODAY()-7</f>
-        <v>46294</v>
+        <v>46296</v>
       </c>
       <c r="S8">
         <f ca="1">DAY(Q8)</f>
-        <v>29</v>
+        <v>1</v>
       </c>
       <c r="T8">
         <f ca="1">MONTH(Q8)</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="U8">
         <f ca="1">YEAR(Q8)</f>

</xml_diff>